<commit_message>
feat: update dataset files and add pelayanan.py script for registration automation
</commit_message>
<xml_diff>
--- a/dataset/dewasa.xlsx
+++ b/dataset/dewasa.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="0" showVerticalScroll="0" showSheetTabs="0" xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="0" showVerticalScroll="0" showSheetTabs="0" xWindow="0" yWindow="780" windowWidth="36000" windowHeight="20940" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -816,7 +816,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:GJ19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" outlineLevelCol="0"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
     <col width="12.6640625" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
@@ -15901,218 +15901,1844 @@
       </c>
     </row>
     <row r="17" ht="17" customHeight="1">
-      <c r="F17" s="9" t="n"/>
-      <c r="H17" s="1" t="n"/>
-      <c r="I17" s="1" t="n"/>
-      <c r="J17" s="1" t="n"/>
-      <c r="BS17" s="9" t="n"/>
-      <c r="BT17" s="9" t="n"/>
-      <c r="BU17" s="9" t="n"/>
-      <c r="BW17" s="9" t="n"/>
-      <c r="BX17" s="9" t="n"/>
-      <c r="BY17" s="9" t="n"/>
-      <c r="BZ17" s="9" t="n"/>
-      <c r="CA17" s="9" t="n"/>
-      <c r="CD17" s="9" t="n"/>
-      <c r="CE17" s="9" t="n"/>
-      <c r="CF17" s="9" t="n"/>
-      <c r="CG17" s="9" t="n"/>
-      <c r="CH17" s="9" t="n"/>
-      <c r="CI17" s="9" t="n"/>
-      <c r="CK17" s="9" t="n"/>
-      <c r="CL17" s="9" t="n"/>
-      <c r="CM17" s="9" t="n"/>
-      <c r="CN17" s="9" t="n"/>
-      <c r="CO17" s="9" t="n"/>
-      <c r="CP17" s="9" t="n"/>
-      <c r="CQ17" s="9" t="n"/>
-      <c r="CS17" s="9" t="n"/>
-      <c r="CT17" s="9" t="n"/>
-      <c r="CU17" s="9" t="n"/>
-      <c r="CV17" s="9" t="n"/>
-      <c r="CX17" s="9" t="n"/>
-      <c r="CY17" s="9" t="n"/>
-      <c r="DA17" s="9" t="n"/>
-      <c r="DB17" s="9" t="n"/>
-      <c r="DD17" s="9" t="n"/>
-      <c r="DF17" s="9" t="n"/>
-      <c r="DG17" s="9" t="n"/>
-      <c r="DH17" s="9" t="n"/>
-      <c r="DI17" s="9" t="n"/>
-      <c r="DJ17" s="9" t="n"/>
-      <c r="DK17" s="9" t="n"/>
-      <c r="DL17" s="9" t="n"/>
-      <c r="DM17" s="9" t="n"/>
-      <c r="DN17" s="9" t="n"/>
-      <c r="DO17" s="9" t="n"/>
-      <c r="DQ17" s="9" t="n"/>
-      <c r="DR17" s="9" t="n"/>
-      <c r="DT17" s="9" t="n"/>
-      <c r="DU17" s="9" t="n"/>
-      <c r="DW17" s="9" t="n"/>
-      <c r="DX17" s="9" t="n"/>
-      <c r="DY17" s="9" t="n"/>
-      <c r="DZ17" s="9" t="n"/>
-      <c r="EA17" s="9" t="n"/>
-      <c r="EB17" s="9" t="n"/>
-      <c r="ED17" s="9" t="n"/>
-      <c r="EF17" s="9" t="n"/>
-      <c r="EG17" s="9" t="n"/>
-      <c r="EH17" s="9" t="n"/>
-      <c r="EI17" s="9" t="n"/>
-      <c r="EK17" s="9" t="n"/>
-      <c r="EL17" s="9" t="n"/>
-      <c r="EN17" s="9" t="n"/>
-      <c r="EO17" s="9" t="n"/>
-      <c r="EP17" s="9" t="n"/>
-      <c r="ER17" s="10" t="n"/>
-      <c r="ES17" s="9" t="n"/>
-      <c r="ET17" s="9" t="n"/>
-      <c r="EU17" s="9" t="n"/>
-      <c r="EW17" s="9" t="n"/>
-      <c r="EX17" s="9" t="n"/>
-      <c r="EY17" s="9" t="n"/>
-      <c r="EZ17" s="9" t="n"/>
-      <c r="FA17" s="9" t="n"/>
-      <c r="FB17" s="9" t="n"/>
-      <c r="FC17" s="9" t="n"/>
-      <c r="FD17" s="9" t="n"/>
-      <c r="FE17" s="9" t="n"/>
-      <c r="FF17" s="9" t="n"/>
-      <c r="FG17" s="9" t="n"/>
-      <c r="FH17" s="9" t="n"/>
-      <c r="FI17" s="9" t="n"/>
-      <c r="FJ17" s="9" t="n"/>
-      <c r="FK17" s="9" t="n"/>
-      <c r="FM17" s="9" t="n"/>
-      <c r="FN17" s="9" t="n"/>
-      <c r="FP17" s="9" t="n"/>
-      <c r="FQ17" s="9" t="n"/>
-      <c r="FR17" s="9" t="n"/>
-      <c r="FT17" s="9" t="n"/>
-      <c r="FU17" s="9" t="n"/>
-      <c r="FV17" s="9" t="n"/>
-      <c r="FW17" s="9" t="n"/>
-      <c r="FX17" s="9" t="n"/>
-      <c r="FY17" s="9" t="n"/>
-      <c r="FZ17" s="9" t="n"/>
-      <c r="GA17" s="9" t="n"/>
-      <c r="GB17" s="9" t="n"/>
-      <c r="GC17" s="9" t="n"/>
-      <c r="GD17" s="9" t="n"/>
-      <c r="GE17" s="9" t="n"/>
-      <c r="GF17" s="9" t="n"/>
-      <c r="GG17" s="9" t="n"/>
-      <c r="GH17" s="9" t="n"/>
-      <c r="GI17" s="9" t="n"/>
-      <c r="GJ17" s="9" t="n"/>
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>ABDUR RAHMAN LATIF</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="I17" s="1" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="J17" s="1" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="K17" s="1" t="inlineStr">
+        <is>
+          <t>Non disabilitas</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="O17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak batuk</t>
+        </is>
+      </c>
+      <c r="Q17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="R17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="S17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="V17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="W17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="X17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="Y17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="Z17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AA17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="AB17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AC17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="AD17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak sama sekali</t>
+        </is>
+      </c>
+      <c r="AE17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak sama sekali</t>
+        </is>
+      </c>
+      <c r="AF17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak sama sekali</t>
+        </is>
+      </c>
+      <c r="AG17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak sama sekali</t>
+        </is>
+      </c>
+      <c r="AH17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="AI17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AJ17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AK17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AL17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AM17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AN17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AO17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="AP17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AQ17" s="4" t="inlineStr">
+        <is>
+          <t>Rokok elektronik (vape, IQOS, dll)</t>
+        </is>
+      </c>
+      <c r="AR17" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS17" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="AT17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AU17" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="AV17" s="4" t="inlineStr">
+        <is>
+          <t>14 s.d &lt;10 tahun lalu</t>
+        </is>
+      </c>
+      <c r="AW17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AX17" s="4" t="inlineStr">
+        <is>
+          <t>Pernah imunisasi tetanus minimal dua kali</t>
+        </is>
+      </c>
+      <c r="AY17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="AZ17" s="4" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="BA17" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB17" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="BC17" s="4" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="BD17" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="BE17" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="BF17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="BG17" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BH17" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="BI17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="BJ17" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="BK17" s="4" t="n">
+        <v>113</v>
+      </c>
+      <c r="BL17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="BM17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN17" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="BO17" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="BP17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ17" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="BR17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="BS17" s="9" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="BT17" s="9" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="BU17" s="9" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="BV17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="BW17" s="5" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="BX17" s="5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="BY17" s="5" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="BZ17" s="5" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="CA17" s="5" t="inlineStr">
+        <is>
+          <t>162</t>
+        </is>
+      </c>
+      <c r="CB17" s="5" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="CC17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="CD17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="CE17" s="5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="CF17" s="9" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="CG17" s="9" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="CH17" s="9" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="CI17" s="9" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="CJ17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="CK17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak batuk</t>
+        </is>
+      </c>
+      <c r="CL17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="CM17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="CN17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="CO17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="CP17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="CQ17" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="CR17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="CS17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak ada</t>
+        </is>
+      </c>
+      <c r="CT17" s="5" t="inlineStr">
+        <is>
+          <t>Bakteriologis</t>
+        </is>
+      </c>
+      <c r="CU17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak dilakukan</t>
+        </is>
+      </c>
+      <c r="CV17" s="5" t="inlineStr">
+        <is>
+          <t>Mtb not detected (Neg)</t>
+        </is>
+      </c>
+      <c r="CW17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="CX17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak Ada</t>
+        </is>
+      </c>
+      <c r="CY17" s="5" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
+      <c r="CZ17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DA17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak Ada</t>
+        </is>
+      </c>
+      <c r="DB17" s="5" t="inlineStr">
+        <is>
+          <t>Bukan kusta</t>
+        </is>
+      </c>
+      <c r="DC17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DD17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak Ada</t>
+        </is>
+      </c>
+      <c r="DE17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DF17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak ada serumen impaksi</t>
+        </is>
+      </c>
+      <c r="DG17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak ada infeksi telinga</t>
+        </is>
+      </c>
+      <c r="DH17" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="DI17" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="DJ17" s="5" t="inlineStr">
+        <is>
+          <t>Normal (visus 6/6 - 6/12)</t>
+        </is>
+      </c>
+      <c r="DK17" s="5" t="inlineStr">
+        <is>
+          <t>Normal (visus 6/6 - 6/12)</t>
+        </is>
+      </c>
+      <c r="DL17" s="5" t="inlineStr">
+        <is>
+          <t>Visus membaik</t>
+        </is>
+      </c>
+      <c r="DM17" s="5" t="inlineStr">
+        <is>
+          <t>Kelainan refraksi ringan (0.50 - 3.00 Dioptri)</t>
+        </is>
+      </c>
+      <c r="DN17" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="DO17" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="DP17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DQ17" s="5" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DR17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="DS17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DT17" s="5" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DU17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="DV17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DW17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="DX17" s="5" t="inlineStr">
+        <is>
+          <t>&lt;20 bungkus per tahun</t>
+        </is>
+      </c>
+      <c r="DY17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="DZ17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="EA17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="EB17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="EC17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="ED17" s="5" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="EE17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="EF17" s="9" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="EG17" s="9" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="EH17" s="9" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="EI17" s="9" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="EJ17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="EK17" s="5" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="EL17" s="5" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="EM17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="EN17" s="5" t="inlineStr">
+        <is>
+          <t>HBsAg Non Reaktif</t>
+        </is>
+      </c>
+      <c r="EO17" s="5" t="inlineStr">
+        <is>
+          <t>Anti HCV Non Reaktif</t>
+        </is>
+      </c>
+      <c r="EP17" s="5" t="inlineStr">
+        <is>
+          <t>VL HCV RNA Negatif</t>
+        </is>
+      </c>
+      <c r="EQ17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="ER17" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="ES17" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="ET17" s="9" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="EU17" s="9" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="EV17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="EW17" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="EX17" s="5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="EY17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="EZ17" s="5" t="inlineStr">
+        <is>
+          <t>SADANIS</t>
+        </is>
+      </c>
+      <c r="FA17" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="FB17" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="FC17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="FD17" s="5" t="inlineStr">
+        <is>
+          <t>HPV Negatif</t>
+        </is>
+      </c>
+      <c r="FE17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="FF17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="FG17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="FH17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="FI17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="FJ17" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="FK17" s="5" t="inlineStr">
+        <is>
+          <t>Negatif</t>
+        </is>
+      </c>
+      <c r="FL17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="FM17" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="FN17" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="FO17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="FP17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak tahu</t>
+        </is>
+      </c>
+      <c r="FQ17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak ditemukan benjolan</t>
+        </is>
+      </c>
+      <c r="FR17" s="5" t="inlineStr">
+        <is>
+          <t>Negatif</t>
+        </is>
+      </c>
+      <c r="FS17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="FT17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak pernah didiagnosis menderita kanker</t>
+        </is>
+      </c>
+      <c r="FU17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak ada keluarga yang terdiagnosis kanker</t>
+        </is>
+      </c>
+      <c r="FV17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak pernah merokok</t>
+        </is>
+      </c>
+      <c r="FW17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak tempat kerja mengandung zat karsinogenik</t>
+        </is>
+      </c>
+      <c r="FX17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak memiliki tempat tinggal berpotensi tinggi</t>
+        </is>
+      </c>
+      <c r="FY17" s="5" t="inlineStr">
+        <is>
+          <t>Memiliki lingkungan dalam rumah yang sehat</t>
+        </is>
+      </c>
+      <c r="FZ17" s="5" t="inlineStr">
+        <is>
+          <t>Tidak pernah didiagnosis penyakit paru kronik</t>
+        </is>
+      </c>
+      <c r="GA17" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="GB17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="GC17" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="GD17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="GE17" s="5" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
+      <c r="GF17" s="5" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
+      <c r="GG17" s="5" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
+      <c r="GH17" s="5" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
+      <c r="GI17" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="GJ17" s="5" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="17" customHeight="1">
-      <c r="F18" s="9" t="n"/>
-      <c r="H18" s="1" t="n"/>
-      <c r="I18" s="1" t="n"/>
-      <c r="J18" s="1" t="n"/>
-      <c r="BS18" s="9" t="n"/>
-      <c r="BT18" s="9" t="n"/>
-      <c r="BU18" s="9" t="n"/>
-      <c r="BW18" s="9" t="n"/>
-      <c r="BX18" s="9" t="n"/>
-      <c r="BY18" s="9" t="n"/>
-      <c r="BZ18" s="9" t="n"/>
-      <c r="CA18" s="9" t="n"/>
-      <c r="CD18" s="9" t="n"/>
-      <c r="CE18" s="9" t="n"/>
-      <c r="CF18" s="9" t="n"/>
-      <c r="CG18" s="9" t="n"/>
-      <c r="CH18" s="9" t="n"/>
-      <c r="CI18" s="9" t="n"/>
-      <c r="CK18" s="9" t="n"/>
-      <c r="CL18" s="9" t="n"/>
-      <c r="CM18" s="9" t="n"/>
-      <c r="CN18" s="9" t="n"/>
-      <c r="CO18" s="9" t="n"/>
-      <c r="CP18" s="9" t="n"/>
-      <c r="CQ18" s="9" t="n"/>
-      <c r="CS18" s="9" t="n"/>
-      <c r="CT18" s="9" t="n"/>
-      <c r="CU18" s="9" t="n"/>
-      <c r="CV18" s="9" t="n"/>
-      <c r="CX18" s="9" t="n"/>
-      <c r="CY18" s="9" t="n"/>
-      <c r="DA18" s="9" t="n"/>
-      <c r="DB18" s="9" t="n"/>
-      <c r="DD18" s="9" t="n"/>
-      <c r="DF18" s="9" t="n"/>
-      <c r="DG18" s="9" t="n"/>
-      <c r="DH18" s="9" t="n"/>
-      <c r="DI18" s="9" t="n"/>
-      <c r="DJ18" s="9" t="n"/>
-      <c r="DK18" s="9" t="n"/>
-      <c r="DL18" s="9" t="n"/>
-      <c r="DM18" s="9" t="n"/>
-      <c r="DN18" s="9" t="n"/>
-      <c r="DO18" s="9" t="n"/>
-      <c r="DQ18" s="9" t="n"/>
-      <c r="DR18" s="9" t="n"/>
-      <c r="DT18" s="9" t="n"/>
-      <c r="DU18" s="9" t="n"/>
-      <c r="DW18" s="9" t="n"/>
-      <c r="DX18" s="9" t="n"/>
-      <c r="DY18" s="9" t="n"/>
-      <c r="DZ18" s="9" t="n"/>
-      <c r="EA18" s="9" t="n"/>
-      <c r="EB18" s="9" t="n"/>
-      <c r="ED18" s="9" t="n"/>
-      <c r="EF18" s="9" t="n"/>
-      <c r="EG18" s="9" t="n"/>
-      <c r="EH18" s="9" t="n"/>
-      <c r="EI18" s="9" t="n"/>
-      <c r="EK18" s="9" t="n"/>
-      <c r="EL18" s="9" t="n"/>
-      <c r="EN18" s="9" t="n"/>
-      <c r="EO18" s="9" t="n"/>
-      <c r="EP18" s="9" t="n"/>
-      <c r="ER18" s="10" t="n"/>
-      <c r="ES18" s="9" t="n"/>
-      <c r="ET18" s="9" t="n"/>
-      <c r="EU18" s="9" t="n"/>
-      <c r="EW18" s="9" t="n"/>
-      <c r="EX18" s="9" t="n"/>
-      <c r="EY18" s="9" t="n"/>
-      <c r="EZ18" s="9" t="n"/>
-      <c r="FA18" s="9" t="n"/>
-      <c r="FB18" s="9" t="n"/>
-      <c r="FC18" s="9" t="n"/>
-      <c r="FD18" s="9" t="n"/>
-      <c r="FE18" s="9" t="n"/>
-      <c r="FF18" s="9" t="n"/>
-      <c r="FG18" s="9" t="n"/>
-      <c r="FH18" s="9" t="n"/>
-      <c r="FI18" s="9" t="n"/>
-      <c r="FJ18" s="9" t="n"/>
-      <c r="FK18" s="9" t="n"/>
-      <c r="FM18" s="9" t="n"/>
-      <c r="FN18" s="9" t="n"/>
-      <c r="FP18" s="9" t="n"/>
-      <c r="FQ18" s="9" t="n"/>
-      <c r="FR18" s="9" t="n"/>
-      <c r="FT18" s="9" t="n"/>
-      <c r="FU18" s="9" t="n"/>
-      <c r="FV18" s="9" t="n"/>
-      <c r="FW18" s="9" t="n"/>
-      <c r="FX18" s="9" t="n"/>
-      <c r="FY18" s="9" t="n"/>
-      <c r="FZ18" s="9" t="n"/>
-      <c r="GA18" s="9" t="n"/>
-      <c r="GB18" s="9" t="n"/>
-      <c r="GC18" s="9" t="n"/>
-      <c r="GD18" s="9" t="n"/>
-      <c r="GE18" s="9" t="n"/>
-      <c r="GF18" s="9" t="n"/>
-      <c r="GG18" s="9" t="n"/>
-      <c r="GH18" s="9" t="n"/>
-      <c r="GI18" s="9" t="n"/>
-      <c r="GJ18" s="9" t="n"/>
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>ADI SASTRO AMIJOYO</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="I18" s="1" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="J18" s="1" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="K18" s="1" t="inlineStr">
+        <is>
+          <t>Non disabilitas</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="O18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="P18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak batuk</t>
+        </is>
+      </c>
+      <c r="Q18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="R18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="T18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="U18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="V18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="W18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="X18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="Y18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="Z18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AA18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="AB18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AC18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="AD18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak sama sekali</t>
+        </is>
+      </c>
+      <c r="AE18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak sama sekali</t>
+        </is>
+      </c>
+      <c r="AF18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak sama sekali</t>
+        </is>
+      </c>
+      <c r="AG18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak sama sekali</t>
+        </is>
+      </c>
+      <c r="AH18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="AI18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AJ18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AK18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AL18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AM18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AN18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AO18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="AP18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AQ18" s="4" t="inlineStr">
+        <is>
+          <t>Rokok elektronik (vape, IQOS, dll)</t>
+        </is>
+      </c>
+      <c r="AR18" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS18" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="AT18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AU18" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="AV18" s="4" t="inlineStr">
+        <is>
+          <t>14 s.d &lt;10 tahun lalu</t>
+        </is>
+      </c>
+      <c r="AW18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="AX18" s="4" t="inlineStr">
+        <is>
+          <t>Pernah imunisasi tetanus minimal dua kali</t>
+        </is>
+      </c>
+      <c r="AY18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="AZ18" s="4" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="BA18" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB18" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="BC18" s="4" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="BD18" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="BE18" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="BF18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="BG18" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BH18" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="BI18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="BJ18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="BK18" s="4" t="n">
+        <v>113</v>
+      </c>
+      <c r="BL18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="BM18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN18" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="BO18" s="4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="BP18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ18" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="BR18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="BS18" s="9" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="BT18" s="9" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="BU18" s="9" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="BV18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="BW18" s="5" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="BX18" s="5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="BY18" s="5" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="BZ18" s="5" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="CA18" s="5" t="inlineStr">
+        <is>
+          <t>162</t>
+        </is>
+      </c>
+      <c r="CB18" s="5" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="CC18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="CD18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="CE18" s="5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="CF18" s="9" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="CG18" s="9" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="CH18" s="9" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="CI18" s="9" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="CJ18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="CK18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak batuk</t>
+        </is>
+      </c>
+      <c r="CL18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="CM18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="CN18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="CO18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="CP18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="CQ18" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="CR18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="CS18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak ada</t>
+        </is>
+      </c>
+      <c r="CT18" s="5" t="inlineStr">
+        <is>
+          <t>Bakteriologis</t>
+        </is>
+      </c>
+      <c r="CU18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak dilakukan</t>
+        </is>
+      </c>
+      <c r="CV18" s="5" t="inlineStr">
+        <is>
+          <t>Mtb not detected (Neg)</t>
+        </is>
+      </c>
+      <c r="CW18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="CX18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak Ada</t>
+        </is>
+      </c>
+      <c r="CY18" s="5" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
+      <c r="CZ18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DA18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak Ada</t>
+        </is>
+      </c>
+      <c r="DB18" s="5" t="inlineStr">
+        <is>
+          <t>Bukan kusta</t>
+        </is>
+      </c>
+      <c r="DC18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DD18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak Ada</t>
+        </is>
+      </c>
+      <c r="DE18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DF18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak ada serumen impaksi</t>
+        </is>
+      </c>
+      <c r="DG18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak ada infeksi telinga</t>
+        </is>
+      </c>
+      <c r="DH18" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="DI18" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="DJ18" s="5" t="inlineStr">
+        <is>
+          <t>Normal (visus 6/6 - 6/12)</t>
+        </is>
+      </c>
+      <c r="DK18" s="5" t="inlineStr">
+        <is>
+          <t>Normal (visus 6/6 - 6/12)</t>
+        </is>
+      </c>
+      <c r="DL18" s="5" t="inlineStr">
+        <is>
+          <t>Visus membaik</t>
+        </is>
+      </c>
+      <c r="DM18" s="5" t="inlineStr">
+        <is>
+          <t>Kelainan refraksi ringan (0.50 - 3.00 Dioptri)</t>
+        </is>
+      </c>
+      <c r="DN18" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="DO18" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="DP18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DQ18" s="5" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DR18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="DS18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DT18" s="5" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DU18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="DV18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="DW18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="DX18" s="5" t="inlineStr">
+        <is>
+          <t>&lt;20 bungkus per tahun</t>
+        </is>
+      </c>
+      <c r="DY18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="DZ18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="EA18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="EB18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="EC18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="ED18" s="5" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="EE18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="EF18" s="9" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="EG18" s="9" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="EH18" s="9" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="EI18" s="9" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="EJ18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="EK18" s="5" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="EL18" s="5" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="EM18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="EN18" s="5" t="inlineStr">
+        <is>
+          <t>HBsAg Non Reaktif</t>
+        </is>
+      </c>
+      <c r="EO18" s="5" t="inlineStr">
+        <is>
+          <t>Anti HCV Non Reaktif</t>
+        </is>
+      </c>
+      <c r="EP18" s="5" t="inlineStr">
+        <is>
+          <t>VL HCV RNA Negatif</t>
+        </is>
+      </c>
+      <c r="EQ18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="ER18" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="ES18" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="ET18" s="9" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="EU18" s="9" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="EV18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="EW18" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="EX18" s="5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="EY18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="EZ18" s="5" t="inlineStr">
+        <is>
+          <t>SADANIS</t>
+        </is>
+      </c>
+      <c r="FA18" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="FB18" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="FC18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="FD18" s="5" t="inlineStr">
+        <is>
+          <t>HPV Negatif</t>
+        </is>
+      </c>
+      <c r="FE18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="FF18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="FG18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="FH18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="FI18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="FJ18" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="FK18" s="5" t="inlineStr">
+        <is>
+          <t>Negatif</t>
+        </is>
+      </c>
+      <c r="FL18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="FM18" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="FN18" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="FO18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="FP18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak tahu</t>
+        </is>
+      </c>
+      <c r="FQ18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak ditemukan benjolan</t>
+        </is>
+      </c>
+      <c r="FR18" s="5" t="inlineStr">
+        <is>
+          <t>Negatif</t>
+        </is>
+      </c>
+      <c r="FS18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="FT18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak pernah didiagnosis menderita kanker</t>
+        </is>
+      </c>
+      <c r="FU18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak ada keluarga yang terdiagnosis kanker</t>
+        </is>
+      </c>
+      <c r="FV18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak pernah merokok</t>
+        </is>
+      </c>
+      <c r="FW18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak tempat kerja mengandung zat karsinogenik</t>
+        </is>
+      </c>
+      <c r="FX18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak memiliki tempat tinggal berpotensi tinggi</t>
+        </is>
+      </c>
+      <c r="FY18" s="5" t="inlineStr">
+        <is>
+          <t>Memiliki lingkungan dalam rumah yang sehat</t>
+        </is>
+      </c>
+      <c r="FZ18" s="5" t="inlineStr">
+        <is>
+          <t>Tidak pernah didiagnosis penyakit paru kronik</t>
+        </is>
+      </c>
+      <c r="GA18" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="GB18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="GC18" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="GD18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="GE18" s="5" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
+      <c r="GF18" s="5" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
+      <c r="GG18" s="5" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
+      <c r="GH18" s="5" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
+      <c r="GI18" s="8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="GJ18" s="5" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="17" customHeight="1">
       <c r="H19" s="1" t="n"/>
@@ -16226,13 +17852,13 @@
     <dataValidation sqref="H2:H19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G16 I2:J19 L2:N16 M17:N19 O2:O19 Q2:T16 R17:T19 U2:AC19 AH2:AJ16 AI17:AJ19 AK2:AP19 AT2:AT19 AW2:AW19 AY2:AY16 AZ2:AZ19 BC2:BC19 BF2:BF19 BI2:BI19 BL2:BL19 BO2:BO19 BR2:BR16 BV2:BV16 BW2:BW19 CC2:CC16 CD2:CD19 CJ2:CJ16 CL2:CP19 CR2:CR16 CW2:CW16 CZ2:CZ16 DC2:DC16 DE2:DE16 DP2:DP16 DQ2:DR19 DS2:DS16 DT2:DU19 DV2:DV16 DY2:EB19 EC2:EC16 EE2:EE16 EJ2:EJ16 EM2:EM16 EQ2:EQ16 EV2:EV16 EY2:EY16 FC2:FC16 FE2:FI19 FL2:FL16 FO2:FO16 FS2:FS16 GB2:GB16 GD2:GD16 GI2:GI16" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G18 I2:J19 L2:N18 M19:N19 O2:O19 Q2:T18 R19:T19 U2:AC19 AH2:AJ18 AI19:AJ19 AK2:AP19 AT2:AT19 AW2:AW19 AY2:AY18 AZ2:AZ19 BC2:BC19 BF2:BF19 BI2:BI19 BL2:BL19 BO2:BO19 BR2:BR18 BV2:BV18 BW2:BW19 CC2:CC18 CD2:CD19 CJ2:CJ18 CL2:CP19 CR2:CR18 CW2:CW18 CZ2:CZ18 DC2:DC18 DE2:DE18 DP2:DP18 DQ2:DR19 DS2:DS18 DT2:DU19 DV2:DV18 DY2:EB19 EC2:EC18 EE2:EE18 EJ2:EJ18 EM2:EM18 EQ2:EQ18 EV2:EV18 EY2:EY18 FC2:FC18 FE2:FI19 FL2:FL18 FO2:FO18 FS2:FS18 GB2:GB18 GD2:GD18 GI2:GI18" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K19 L17:L19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K19 L19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation sqref="AD2:AG19 AH17:AH19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="AD2:AG19 AH19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Tidak sama sekali,Kurang dari 1 minggu,Lebih dari 1 minggu,Hampir setiap hari"</formula1>
     </dataValidation>
     <dataValidation sqref="AV2:AV19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -16253,7 +17879,7 @@
     <dataValidation sqref="CX2:CX19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation sqref="CY2:CY19 GE2:GH19 GI17:GI19 GJ2:GJ19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="CY2:CY19 GE2:GH19 GI19 GJ2:GJ19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
     <dataValidation sqref="DA2:DA19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -16340,7 +17966,7 @@
     <dataValidation sqref="FY2:FY19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation sqref="GA2:GA19 GB17:GB19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="GA2:GA19 GB19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
     <dataValidation sqref="EZ2:EZ19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -16349,7 +17975,7 @@
     <dataValidation sqref="FA2:FA19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Normal,Ditemukan benjolan,Curiga kanker"</formula1>
     </dataValidation>
-    <dataValidation sqref="FB2:FB19 FC17:FC19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="FB2:FB19 FC19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>" Normal,Simple cyst,Non simple cyst"</formula1>
     </dataValidation>
     <dataValidation sqref="FD2:FD19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -16358,10 +17984,10 @@
     <dataValidation sqref="FJ2:FJ19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Normal,Curiga kanker"</formula1>
     </dataValidation>
-    <dataValidation sqref="AX2:AX19 AY17:AY19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="AX2:AX19 AY19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Pernah imunisasi tetanus minimal dua kali,Pernah imunisasi tetanus satu kali,Pernah imunisasi tetanus tetapi tidak ingat berapa kali,Tidak tahu atau tidak ingat"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P19 Q17:Q19 AQ2:AQ19 CK2:CK19 CV2:CV19 FW2:FW19 FZ2:FZ19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list"/>
+    <dataValidation sqref="P2:P19 Q19 AQ2:AQ19 CK2:CK19 CV2:CV19 FW2:FW19 FZ2:FZ19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>